<commit_message>
Added RAD Motor Fuel Lice Number Test Cases and updated scripts from Selenium to WebDriver
</commit_message>
<xml_diff>
--- a/KatalonData/RADTestData/CRNNotZero.xlsx
+++ b/KatalonData/RADTestData/CRNNotZero.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\t465179\Documents\git\VPS-Katalon\VPS-Katalon\KatalonData\RADTestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B564D908-B342-473F-9B0B-E3C78161EF4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E34750F-9142-4614-9618-F9E0F613FB58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" xr2:uid="{D99FAB39-5CE6-4AA4-B9C6-99B1EFA0654E}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="CRNNotZero" sheetId="4" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">CRNNotZero!$E$1:$E$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">CRNNotZero!$E$1:$E$11</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="24">
   <si>
     <t>Result</t>
   </si>
@@ -486,7 +486,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3B7105E-5E71-456F-8D2A-C4C503B29111}">
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr defaultColWidth="9.19921875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="9.19921875" style="1" collapsed="1"/>
@@ -687,16 +687,20 @@
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A12"/>
-      <c r="B12"/>
+      <c r="A12" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12" t="s">
+        <v>23</v>
+      </c>
       <c r="C12" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="F12" s="1" t="s">
         <v>11</v>
@@ -709,10 +713,10 @@
         <v>11</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F13" s="1" t="s">
         <v>11</v>
@@ -725,10 +729,10 @@
         <v>11</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F14" s="1" t="s">
         <v>11</v>
@@ -741,10 +745,10 @@
         <v>11</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F15" s="1" t="s">
         <v>11</v>
@@ -757,10 +761,10 @@
         <v>11</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F16" s="1" t="s">
         <v>11</v>
@@ -773,10 +777,10 @@
         <v>11</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="F17" s="1" t="s">
         <v>11</v>
@@ -789,341 +793,17 @@
         <v>11</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F18" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A19"/>
-      <c r="B19"/>
-      <c r="C19" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="E19" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A20"/>
-      <c r="B20"/>
-      <c r="C20" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A21"/>
-      <c r="B21"/>
-      <c r="C21" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="F21" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A22"/>
-      <c r="B22"/>
-      <c r="C22" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="E22" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F22" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A23"/>
-      <c r="B23"/>
-      <c r="C23" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F23" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A24"/>
-      <c r="B24"/>
-      <c r="C24" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="E24" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F24" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A25"/>
-      <c r="B25"/>
-      <c r="C25" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="E25" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="F25" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A26"/>
-      <c r="B26"/>
-      <c r="C26" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="E26" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F26" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A27"/>
-      <c r="B27"/>
-      <c r="C27" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="E27" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F27" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A28"/>
-      <c r="B28"/>
-      <c r="C28" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="E28" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="F28" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A29"/>
-      <c r="B29"/>
-      <c r="C29" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D29" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="E29" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F29" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A30"/>
-      <c r="B30"/>
-      <c r="C30" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="E30" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="F30" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A31"/>
-      <c r="B31"/>
-      <c r="C31" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D31" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="E31" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="F31" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A32" t="s">
-        <v>20</v>
-      </c>
-      <c r="B32" t="s">
-        <v>23</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D32" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E32" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="F32" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A33"/>
-      <c r="B33"/>
-      <c r="C33" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E33" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F33" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A34"/>
-      <c r="B34"/>
-      <c r="C34" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D34" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E34" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="F34" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A35"/>
-      <c r="B35"/>
-      <c r="C35" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D35" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E35" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F35" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A36"/>
-      <c r="B36"/>
-      <c r="C36" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D36" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E36" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F36" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A37"/>
-      <c r="B37"/>
-      <c r="C37" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D37" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E37" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="F37" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A38"/>
-      <c r="B38"/>
-      <c r="C38" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D38" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E38" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F38" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="E1:E31" xr:uid="{E3B7105E-5E71-456F-8D2A-C4C503B29111}"/>
+  <autoFilter ref="E1:E11" xr:uid="{E3B7105E-5E71-456F-8D2A-C4C503B29111}"/>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>

</xml_diff>